<commit_message>
Non-metro routes: capture every flight across all airlines
- DEL-JAI and PNQ-BLR now use mode='all': show every nonstop flight and
  every airline (Air India, Alliance Air, Air India Express, Akasa, IndiGo),
  not IndiGo-only 3-slot view
- Refactored render to entries-per-sector supporting slots + all modes
- Handle null-price flights (e.g. Alliance Air in Google Flights)
- Excel 'Tracked flights' sheet and trend charts follow the same entries

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fares.xlsx
+++ b/fares.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="All fares" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Slot view" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tracked flights" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25760,12 +25760,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
@@ -25792,7 +25792,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>slot</t>
+          <t>row</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -25929,31 +25929,31 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>Morning</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>D+1</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>AI 2803</t>
+          <t>AI 427</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>13670</v>
+        <v>10226</v>
       </c>
     </row>
     <row r="5">
@@ -25979,12 +25979,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -25998,7 +25998,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>10226</v>
+        <v>10121</v>
       </c>
     </row>
     <row r="6">
@@ -26019,31 +26019,31 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Morning</t>
+          <t>Evening</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>+3wk</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>AI 427</t>
+          <t>AI 2487</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>10121</v>
+        <v>15376</v>
       </c>
     </row>
     <row r="7">
@@ -26064,31 +26064,31 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Morning</t>
+          <t>Evening</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>D+1</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>AI 427</t>
+          <t>AI 2487</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>12867</v>
+        <v>10226</v>
       </c>
     </row>
     <row r="8">
@@ -26104,12 +26104,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>Early morning</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -26124,16 +26124,16 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>07:05</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>AI 2487</t>
+          <t>6E 810</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>15376</v>
+        <v>10096</v>
       </c>
     </row>
     <row r="9">
@@ -26149,12 +26149,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>Early morning</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -26169,16 +26169,16 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>07:05</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>AI 2487</t>
+          <t>6E 810</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>10226</v>
+        <v>10096</v>
       </c>
     </row>
     <row r="10">
@@ -26194,36 +26194,36 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>Morning</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>D+1</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>AI 2487</t>
+          <t>6E 826</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>11433</v>
+        <v>10096</v>
       </c>
     </row>
     <row r="11">
@@ -26244,31 +26244,31 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>Morning</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>07:05</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>6E 810</t>
+          <t>6E 826</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>10096</v>
+        <v>9795</v>
       </c>
     </row>
     <row r="12">
@@ -26289,31 +26289,31 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>Evening</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>+3wk</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>07:05</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>6E 810</t>
+          <t>6E 811</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>10096</v>
+        <v>11603</v>
       </c>
     </row>
     <row r="13">
@@ -26334,31 +26334,31 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>Evening</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>D+1</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>07:05</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>6E 810</t>
+          <t>6E 811</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>13365</v>
+        <v>10096</v>
       </c>
     </row>
     <row r="14">
@@ -26369,17 +26369,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Delhi → Bengaluru</t>
+          <t>Delhi → Jaipur</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Morning</t>
+          <t>AI 1767</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -26394,16 +26394,16 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>6E 826</t>
+          <t>AI 1767</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>10096</v>
+        <v>4533</v>
       </c>
     </row>
     <row r="15">
@@ -26414,17 +26414,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Delhi → Bengaluru</t>
+          <t>Delhi → Jaipur</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Morning</t>
+          <t>AI 1767</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -26439,16 +26439,16 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>6E 826</t>
+          <t>AI 1767</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>9795</v>
+        <v>4533</v>
       </c>
     </row>
     <row r="16">
@@ -26459,41 +26459,41 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Delhi → Bengaluru</t>
+          <t>Delhi → Jaipur</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Morning</t>
+          <t>AI 429</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>D+1</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:20</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>6E 826</t>
+          <t>AI 429</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>12160</v>
+        <v>13489</v>
       </c>
     </row>
     <row r="17">
@@ -26504,17 +26504,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Delhi → Bengaluru</t>
+          <t>Delhi → Jaipur</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Alliance Air</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>9I 843</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -26529,16 +26529,13 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>6E 811</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>11603</v>
+          <t>9I 843</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -26549,17 +26546,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Delhi → Bengaluru</t>
+          <t>Delhi → Jaipur</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Alliance Air</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>9I 843</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -26574,16 +26571,13 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>6E 811</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>10096</v>
+          <t>9I 843</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -26594,7 +26588,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Delhi → Bengaluru</t>
+          <t>Delhi → Jaipur</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -26604,31 +26598,31 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>6E 6190</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>D+1</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>07:40</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>6E 811</t>
+          <t>6E 6190</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>11075</v>
+        <v>3220</v>
       </c>
     </row>
     <row r="20">
@@ -26644,36 +26638,36 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>6E 6190</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:40</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>AI 1767</t>
+          <t>6E 6190</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>4533</v>
+        <v>4795</v>
       </c>
     </row>
     <row r="21">
@@ -26689,36 +26683,36 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>6E 5033</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>+3wk</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>AI 1767</t>
+          <t>6E 5033</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>4533</v>
+        <v>5320</v>
       </c>
     </row>
     <row r="22">
@@ -26734,36 +26728,36 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Morning</t>
+          <t>6E 5033</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>15:50</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>AI 1767</t>
+          <t>6E 5033</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>4533</v>
+        <v>3010</v>
       </c>
     </row>
     <row r="23">
@@ -26779,36 +26773,36 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Morning</t>
+          <t>6E 6131</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>+3wk</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>20:20</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>AI 429</t>
+          <t>6E 6131</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>13489</v>
+        <v>5845</v>
       </c>
     </row>
     <row r="24">
@@ -26829,27 +26823,27 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>6E 6131</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>07:40</t>
+          <t>20:20</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>6E 6190</t>
+          <t>6E 6131</t>
         </is>
       </c>
       <c r="I24" t="n">
@@ -26864,12 +26858,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Delhi → Jaipur</t>
+          <t>Delhi → Mumbai</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -26879,26 +26873,26 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>+3wk</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>07:40</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>6E 6190</t>
+          <t>AI 2975</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>4795</v>
+        <v>7170</v>
       </c>
     </row>
     <row r="26">
@@ -26909,41 +26903,41 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Delhi → Jaipur</t>
+          <t>Delhi → Mumbai</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Morning</t>
+          <t>Early morning</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>07:40</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>6E 6190</t>
+          <t>AI 2975</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>3220</v>
+        <v>7433</v>
       </c>
     </row>
     <row r="27">
@@ -26954,12 +26948,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Delhi → Jaipur</t>
+          <t>Delhi → Mumbai</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -26969,26 +26963,26 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>+3wk</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>07:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>6E 6190</t>
+          <t>AI 2963</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>4795</v>
+        <v>7433</v>
       </c>
     </row>
     <row r="28">
@@ -26999,41 +26993,41 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Delhi → Jaipur</t>
+          <t>Delhi → Mumbai</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>Morning</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>6E 6131</t>
+          <t>AI 2963</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>5845</v>
+        <v>7170</v>
       </c>
     </row>
     <row r="29">
@@ -27044,12 +27038,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Delhi → Jaipur</t>
+          <t>Delhi → Mumbai</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -27059,26 +27053,26 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>+3wk</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>6E 6131</t>
+          <t>AI 2955</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>3220</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="30">
@@ -27099,27 +27093,27 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>Evening</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>AI 2975</t>
+          <t>AI 2441</t>
         </is>
       </c>
       <c r="I30" t="n">
@@ -27139,7 +27133,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -27149,26 +27143,26 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>+3wk</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:05</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>AI 2975</t>
+          <t>6E 6218</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>7433</v>
+        <v>7225</v>
       </c>
     </row>
     <row r="32">
@@ -27184,7 +27178,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -27194,26 +27188,26 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>D+1</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:05</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>AI 2975</t>
+          <t>6E 6218</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>7170</v>
+        <v>6963</v>
       </c>
     </row>
     <row r="33">
@@ -27229,7 +27223,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -27249,16 +27243,16 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>AI 2963</t>
+          <t>6E 675</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>7433</v>
+        <v>7225</v>
       </c>
     </row>
     <row r="34">
@@ -27274,7 +27268,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -27294,16 +27288,16 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>AI 2963</t>
+          <t>6E 675</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>7170</v>
+        <v>6963</v>
       </c>
     </row>
     <row r="35">
@@ -27319,36 +27313,36 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Morning</t>
+          <t>Evening</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>D+1</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>AI 2963</t>
+          <t>6E 329</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>7170</v>
+        <v>7593</v>
       </c>
     </row>
     <row r="36">
@@ -27364,7 +27358,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>IndiGo</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -27374,12 +27368,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -27389,11 +27383,11 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>AI 2955</t>
+          <t>6E 329</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>8000</v>
+        <v>7225</v>
       </c>
     </row>
     <row r="37">
@@ -27404,41 +27398,41 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Delhi → Mumbai</t>
+          <t>Pune → Bengaluru</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>Air India Express</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>IX 2681</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>+3wk</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>AI 2441</t>
+          <t>IX 2681</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>7170</v>
+        <v>5536</v>
       </c>
     </row>
     <row r="38">
@@ -27449,41 +27443,41 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Delhi → Mumbai</t>
+          <t>Pune → Bengaluru</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Air India</t>
+          <t>Air India Express</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>IX 2681</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>D+1</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>00:05</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>AI 2955</t>
+          <t>IX 2681</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>7170</v>
+        <v>5536</v>
       </c>
     </row>
     <row r="39">
@@ -27494,41 +27488,41 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Delhi → Mumbai</t>
+          <t>Pune → Bengaluru</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India Express</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>IX 2706</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>06:05</t>
+          <t>05:10</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>6E 6218</t>
+          <t>IX 2706</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>7225</v>
+        <v>5536</v>
       </c>
     </row>
     <row r="40">
@@ -27539,41 +27533,41 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Delhi → Mumbai</t>
+          <t>Pune → Bengaluru</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India Express</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>IX 2706</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>+3wk</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>06:05</t>
+          <t>05:40</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>6E 6218</t>
+          <t>IX 2706</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>6963</v>
+        <v>5536</v>
       </c>
     </row>
     <row r="41">
@@ -27584,41 +27578,41 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Delhi → Mumbai</t>
+          <t>Pune → Bengaluru</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India Express</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>IX 2718</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>D+1</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>06:05</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>6E 6218</t>
+          <t>IX 2718</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>6963</v>
+        <v>5536</v>
       </c>
     </row>
     <row r="42">
@@ -27629,41 +27623,41 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Delhi → Mumbai</t>
+          <t>Pune → Bengaluru</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India Express</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Morning</t>
+          <t>IX 2718</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>6E 675</t>
+          <t>IX 2718</t>
         </is>
       </c>
       <c r="I42" t="n">
-        <v>7225</v>
+        <v>5536</v>
       </c>
     </row>
     <row r="43">
@@ -27674,17 +27668,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Delhi → Mumbai</t>
+          <t>Pune → Bengaluru</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India Express</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Morning</t>
+          <t>IX 2874</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -27699,16 +27693,16 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>6E 675</t>
+          <t>IX 2874</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>6963</v>
+        <v>7555</v>
       </c>
     </row>
     <row r="44">
@@ -27719,41 +27713,41 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Delhi → Mumbai</t>
+          <t>Pune → Bengaluru</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India Express</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Morning</t>
+          <t>IX 2874</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>D+1</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>6E 675</t>
+          <t>IX 2874</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>6963</v>
+        <v>8047</v>
       </c>
     </row>
     <row r="45">
@@ -27764,17 +27758,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Delhi → Mumbai</t>
+          <t>Pune → Bengaluru</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India Express</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>IX 2839</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -27789,16 +27783,16 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>6E 329</t>
+          <t>IX 2839</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>7593</v>
+        <v>6072</v>
       </c>
     </row>
     <row r="46">
@@ -27809,17 +27803,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Delhi → Mumbai</t>
+          <t>Pune → Bengaluru</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Air India Express</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>IX 2839</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -27834,16 +27828,16 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>6E 329</t>
+          <t>IX 2839</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>7225</v>
+        <v>6072</v>
       </c>
     </row>
     <row r="47">
@@ -27854,41 +27848,41 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Delhi → Mumbai</t>
+          <t>Pune → Bengaluru</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Akasa Air</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>QP 1312</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>D+1</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>07:25</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>6E 329</t>
+          <t>QP 1312</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>6963</v>
+        <v>5613</v>
       </c>
     </row>
     <row r="48">
@@ -27904,36 +27898,36 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Akasa Air</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>QP 1312</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>07:25</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>6E 391</t>
+          <t>QP 1312</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>5313</v>
+        <v>5428</v>
       </c>
     </row>
     <row r="49">
@@ -27949,36 +27943,36 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Akasa Air</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Early morning</t>
+          <t>QP 1314</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>+3wk</t>
+          <t>+1wk</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>6E 391</t>
+          <t>QP 1314</t>
         </is>
       </c>
       <c r="I49" t="n">
-        <v>5313</v>
+        <v>7143</v>
       </c>
     </row>
     <row r="50">
@@ -27994,36 +27988,36 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>IndiGo</t>
+          <t>Akasa Air</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Evening</t>
+          <t>QP 1314</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>+1wk</t>
+          <t>+3wk</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>6E 174</t>
+          <t>QP 1314</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>5313</v>
+        <v>5252</v>
       </c>
     </row>
     <row r="51">
@@ -28039,35 +28033,1070 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
+          <t>Akasa Air</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>QP 1326</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>+1wk</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>QP 1326</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>5613</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Akasa Air</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>QP 1326</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>+3wk</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>QP 1326</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>5083</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Akasa Air</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>QP 1316</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>+1wk</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>QP 1316</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>9202</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Akasa Air</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>QP 1316</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>+3wk</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>QP 1316</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>5613</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Akasa Air</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>QP 1318</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>+1wk</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>22:10</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>QP 1318</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>7671</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Akasa Air</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>QP 1318</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>+3wk</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>22:10</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>QP 1318</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>5252</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
           <t>IndiGo</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Evening</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>6E 361</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>+1wk</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>01:15</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>6E 361</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>6E 361</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>+3wk</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>2026-08-14</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>01:15</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>6E 361</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>6E 6564</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>+1wk</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>03:15</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>6E 6564</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>6E 6564</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>+3wk</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>03:15</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>6E 6564</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>6E 6877</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>+1wk</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>6E 6877</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>6E 6877</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>+3wk</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>05:00</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>6E 6877</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>6E 391</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>+1wk</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>06:40</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>6E 391</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>6E 391</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>+3wk</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>06:40</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>6E 391</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>6E 302</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>+1wk</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>6E 302</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>6E 302</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>+3wk</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>6E 302</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>6094</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>6E 137</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>+1wk</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>6E 137</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>6E 137</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>+3wk</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>6E 137</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>6E 174</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>+1wk</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
         <is>
           <t>17:40</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="H69" t="inlineStr">
         <is>
           <t>6E 174</t>
         </is>
       </c>
-      <c r="I51" t="n">
+      <c r="I69" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>6E 174</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>+3wk</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>6E 174</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>6E 107</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>+1wk</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>6E 107</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>6E 107</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>+3wk</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>6E 107</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>6094</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>6E 6055</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>+1wk</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>23:50</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>6E 6055</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>5313</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Pune → Bengaluru</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>IndiGo</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>6E 6055</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>+3wk</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>23:50</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>6E 6055</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
         <v>5313</v>
       </c>
     </row>

</xml_diff>